<commit_message>
Updating profili di consumo blnp
</commit_message>
<xml_diff>
--- a/files/energy/input/load_emulator/input_emulator_v2/3. appliances_load_profiles_v2.xlsx
+++ b/files/energy/input/load_emulator/input_emulator_v2/3. appliances_load_profiles_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rsericerca-my.sharepoint.com/personal/rollo_rse-web_it/Documents/Desktop/CACER simulator - public repo/CACER-simulator/files/energy/input/load_emulator/input_emulator_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="728" documentId="11_6B245526C2F3A0A249C1BFFA6B23B9E3661639BD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FA43219-3CC1-4AFE-8093-7817FB70A60C}"/>
+  <xr:revisionPtr revIDLastSave="744" documentId="11_6B245526C2F3A0A249C1BFFA6B23B9E3661639BD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37E8E190-ECE6-483B-9089-E1EB18691DC2}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="877" firstSheet="40" activeTab="42" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="877" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="blender_1" sheetId="56" r:id="rId1"/>
@@ -220,7 +220,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="178" formatCode="0.00000"/>
+    <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -328,7 +328,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3932,16 +3932,16 @@
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1.271849870953806E-2</v>
+      <c r="B2" s="5">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>2.6575149753164211E-3</v>
+      <c r="B3" s="5">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -60044,7 +60044,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="11">
-        <v>0.20086844404838811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -60052,7 +60052,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="11">
-        <v>5.9083183527890187E-2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -60082,7 +60082,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="11">
-        <v>6.7907526239147104E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -60090,7 +60090,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="11">
-        <v>1.344895905513135E-3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -60120,7 +60120,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="11">
-        <v>6.7308799449090654E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -60128,7 +60128,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="11">
-        <v>1.384650142961614E-3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -60158,7 +60158,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="11">
-        <v>3.0297276585419162E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -60166,7 +60166,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="11">
-        <v>2.2467240589840159E-4</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -75495,7 +75495,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="11">
-        <v>8.3457420097193577E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -75503,7 +75503,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="11">
-        <v>1.082205498735587E-2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -76324,7 +76324,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="11">
-        <v>1.035321947494445E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -76332,7 +76332,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="11">
-        <v>7.6999211696182613E-4</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>